<commit_message>
fix: Logout Handling (No Middleware Yet)
</commit_message>
<xml_diff>
--- a/Diagram/UseCaseDescription.xlsx
+++ b/Diagram/UseCaseDescription.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/paultsai/Desktop/SLC/TPA/Desktop/TPA-Desktop/Diagram/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFB371F4-B3BB-1B46-A87C-4F5B9CF81B83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A50D3A0-03F6-CB4B-8FB5-3B82D6D7C54F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" activeTab="7" xr2:uid="{2183EE87-2FE0-1848-A8EC-EAF6DA5552F2}"/>
+    <workbookView minimized="1" xWindow="-20" yWindow="760" windowWidth="30240" windowHeight="18880" activeTab="7" xr2:uid="{2183EE87-2FE0-1848-A8EC-EAF6DA5552F2}"/>
   </bookViews>
   <sheets>
     <sheet name="1. Add New Menu Item" sheetId="1" r:id="rId1"/>
@@ -1220,7 +1220,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="94">
+  <cellXfs count="93">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1476,9 +1476,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -5301,7 +5298,9 @@
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" s="11"/>
       <c r="B15" s="69"/>
-      <c r="C15" s="93"/>
+      <c r="C15" s="83" t="s">
+        <v>232</v>
+      </c>
       <c r="D15" s="19" t="s">
         <v>190</v>
       </c>
@@ -5309,9 +5308,7 @@
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16" s="11"/>
       <c r="B16" s="69"/>
-      <c r="C16" s="65" t="s">
-        <v>232</v>
-      </c>
+      <c r="C16" s="84"/>
       <c r="D16" s="19" t="s">
         <v>300</v>
       </c>
@@ -5319,7 +5316,7 @@
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" s="11"/>
       <c r="B17" s="69"/>
-      <c r="C17" s="66"/>
+      <c r="C17" s="84"/>
       <c r="D17" s="19" t="s">
         <v>285</v>
       </c>
@@ -5327,7 +5324,7 @@
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" s="11"/>
       <c r="B18" s="70"/>
-      <c r="C18" s="67"/>
+      <c r="C18" s="85"/>
       <c r="D18" s="19" t="s">
         <v>286</v>
       </c>
@@ -5784,13 +5781,13 @@
     <mergeCell ref="C7:D7"/>
     <mergeCell ref="B13:B18"/>
     <mergeCell ref="C20:D20"/>
-    <mergeCell ref="C16:C18"/>
     <mergeCell ref="B19:B20"/>
     <mergeCell ref="C9:D9"/>
     <mergeCell ref="C10:D10"/>
     <mergeCell ref="C11:D11"/>
     <mergeCell ref="C12:D12"/>
     <mergeCell ref="C19:D19"/>
+    <mergeCell ref="C15:C18"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="C3:D3"/>
     <mergeCell ref="B4:B6"/>

</xml_diff>